<commit_message>
Updated acceptance tests and requirements
</commit_message>
<xml_diff>
--- a/G3_Acceptance.Ass1.xlsx
+++ b/G3_Acceptance.Ass1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liorg\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eli\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C532738C-750B-48FA-86BE-B4C0D428D69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDFCD5A5-EE3E-4B68-98A0-39F12A737F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BCB4B167-D6B0-4D98-93B3-2388AFB6BFC1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BCB4B167-D6B0-4D98-93B3-2388AFB6BFC1}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirments" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="197">
   <si>
     <t>Test ID</t>
   </si>
@@ -801,18 +801,6 @@
     </r>
   </si>
   <si>
-    <t>Lior Ginat  - 211879804</t>
-  </si>
-  <si>
-    <t>Anna Papikyan - 324390939</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dor Stern - 322468349 </t>
-  </si>
-  <si>
-    <t>Adi Varshavsky -  209141068</t>
-  </si>
-  <si>
     <t>GROUP #3</t>
   </si>
   <si>
@@ -942,6 +930,66 @@
   </si>
   <si>
     <t>The system cancels their pending spot, frees the space, and (if applicable) sends a notification to the next person on the waiting list.</t>
+  </si>
+  <si>
+    <t>ExitParkSuccess</t>
+  </si>
+  <si>
+    <t>A park employee identifies a departing visitor (by ID or QR code). Clicks: register exit.</t>
+  </si>
+  <si>
+    <t>The system successfully records the exit and decreases the current number of visitors in the park, updating the available capacity.</t>
+  </si>
+  <si>
+    <t>A visitor is currently registered as inside the park</t>
+  </si>
+  <si>
+    <t>Covers req: System allows updates on the number of visitors (decreasing to free up space).</t>
+  </si>
+  <si>
+    <t>RegisterExistingGuide</t>
+  </si>
+  <si>
+    <t>A customer representative logs in. Types the details of a guide who is already registered in the system. Clicks: save.</t>
+  </si>
+  <si>
+    <t>The system prevents the registration and displays an error message stating that the guide is already registered.</t>
+  </si>
+  <si>
+    <t>A customer representative is logged in, and the guide's ID is already in the Database.</t>
+  </si>
+  <si>
+    <t>Attempting to register a guide that already exists</t>
+  </si>
+  <si>
+    <t>UnauthorizedGuideRegistration</t>
+  </si>
+  <si>
+    <t>A regular park employee (not a customer representative) logs in and attempts to navigate to the guide registration screen.</t>
+  </si>
+  <si>
+    <t>The system blocks access to the screen and displays an error message stating: "Unauthorized access: Only a customer representative can register a guide.</t>
+  </si>
+  <si>
+    <t>A park employee is logged into the system</t>
+  </si>
+  <si>
+    <t>Registering a new guide is processed by a customer representative only</t>
+  </si>
+  <si>
+    <t>ליאור גינת - 211879804</t>
+  </si>
+  <si>
+    <t>אנה פפיקיאן - 324390939</t>
+  </si>
+  <si>
+    <t>עדי ורשבסקי -  209141068</t>
+  </si>
+  <si>
+    <t xml:space="preserve">דור שטרן - 322468349 </t>
+  </si>
+  <si>
+    <t>ליאור גינת  - 211879804</t>
   </si>
 </sst>
 </file>
@@ -1749,71 +1797,71 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C232064-FE95-4172-B996-81E675FC027A}">
   <dimension ref="A1:D44"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" style="11" customWidth="1"/>
-    <col min="2" max="2" width="22.59765625" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.625" style="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="61.5" style="11" customWidth="1"/>
-    <col min="4" max="4" width="29.69921875" style="11" customWidth="1"/>
-    <col min="5" max="5" width="16.69921875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="14.19921875" style="11" customWidth="1"/>
+    <col min="4" max="4" width="29.625" style="11" customWidth="1"/>
+    <col min="5" max="5" width="16.625" style="11" customWidth="1"/>
+    <col min="6" max="6" width="14.125" style="11" customWidth="1"/>
     <col min="7" max="7" width="9" style="11"/>
-    <col min="8" max="8" width="6.59765625" style="11" customWidth="1"/>
-    <col min="9" max="9" width="12.69921875" style="11" customWidth="1"/>
+    <col min="8" max="8" width="6.625" style="11" customWidth="1"/>
+    <col min="9" max="9" width="12.625" style="11" customWidth="1"/>
     <col min="10" max="10" width="41.5" style="11" customWidth="1"/>
     <col min="11" max="11" width="21" style="11" customWidth="1"/>
     <col min="12" max="13" width="12.5" style="11" customWidth="1"/>
-    <col min="14" max="14" width="12.19921875" style="11" customWidth="1"/>
+    <col min="14" max="14" width="12.125" style="11" customWidth="1"/>
     <col min="15" max="16384" width="9" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="12" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B1" s="14">
-        <v>46207</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>46330</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C2" s="12" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C3" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C3" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="C4" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C5" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C6" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="D6" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="D4" s="13" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C5" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C6" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:4" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
@@ -1824,14 +1872,14 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B9" s="23" t="s">
         <v>31</v>
       </c>
       <c r="C9" s="24"/>
       <c r="D9" s="25"/>
     </row>
-    <row r="10" spans="1:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="8">
         <v>1</v>
       </c>
@@ -1842,7 +1890,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
         <v>2</v>
       </c>
@@ -1853,7 +1901,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B12" s="6">
         <v>3</v>
       </c>
@@ -1864,7 +1912,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B13" s="6">
         <v>4</v>
       </c>
@@ -1875,7 +1923,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" s="6">
         <v>5</v>
       </c>
@@ -1886,7 +1934,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B15" s="6">
         <v>6</v>
       </c>
@@ -1897,7 +1945,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B16" s="6">
         <v>7</v>
       </c>
@@ -1908,7 +1956,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B17" s="6">
         <v>8</v>
       </c>
@@ -1919,7 +1967,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B18" s="6">
         <v>9</v>
       </c>
@@ -1930,7 +1978,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B19" s="6">
         <v>10</v>
       </c>
@@ -1941,7 +1989,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B20" s="6">
         <v>11</v>
       </c>
@@ -1952,7 +2000,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B21" s="6">
         <v>12</v>
       </c>
@@ -1963,7 +2011,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B22" s="6">
         <v>13</v>
       </c>
@@ -1974,7 +2022,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B23" s="6">
         <v>14</v>
       </c>
@@ -1985,7 +2033,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B24" s="6">
         <v>15</v>
       </c>
@@ -1996,7 +2044,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" s="6">
         <v>16</v>
       </c>
@@ -2007,7 +2055,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B26" s="6">
         <v>17</v>
       </c>
@@ -2018,7 +2066,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B27" s="6">
         <v>18</v>
       </c>
@@ -2029,7 +2077,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B28" s="6">
         <v>19</v>
       </c>
@@ -2040,7 +2088,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B29" s="6">
         <v>20</v>
       </c>
@@ -2051,7 +2099,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B30" s="6">
         <v>21</v>
       </c>
@@ -2062,7 +2110,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B31" s="6">
         <v>22</v>
       </c>
@@ -2073,7 +2121,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:4" ht="30" x14ac:dyDescent="0.2">
       <c r="B32" s="19">
         <v>23</v>
       </c>
@@ -2084,7 +2132,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B33" s="18">
         <v>24</v>
       </c>
@@ -2095,80 +2143,80 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="2:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B34" s="18">
         <v>25</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:4" ht="30" x14ac:dyDescent="0.2">
       <c r="B35" s="18">
         <v>26</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D35" s="18" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:4" ht="30" x14ac:dyDescent="0.2">
       <c r="B36" s="18">
         <v>27</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D36" s="18" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="2:4" ht="15.6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:4" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B37" s="18">
         <v>28</v>
       </c>
       <c r="C37" s="17" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D37" s="18" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="2:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:4" ht="30" x14ac:dyDescent="0.2">
       <c r="B38" s="18">
         <v>29</v>
       </c>
       <c r="C38" s="17" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D38" s="18" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="2:4" ht="15.6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:4" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B39" s="18">
         <v>30</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D39" s="18" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="40" spans="2:4" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B40" s="26" t="s">
         <v>121</v>
       </c>
       <c r="C40" s="27"/>
       <c r="D40" s="28"/>
     </row>
-    <row r="41" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B41" s="6">
         <v>1</v>
       </c>
@@ -2179,7 +2227,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B42" s="6">
         <v>2</v>
       </c>
@@ -2190,7 +2238,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B43" s="6">
         <v>3</v>
       </c>
@@ -2201,7 +2249,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="2:4" ht="30.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B44" s="6">
         <v>4</v>
       </c>
@@ -2230,67 +2278,67 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B354F86-0223-4F72-8EED-E4B6E788A3A6}">
-  <dimension ref="A1:G37"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G40"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" style="10" customWidth="1"/>
     <col min="2" max="2" width="9" style="10"/>
     <col min="3" max="3" width="24.5" style="10" customWidth="1"/>
     <col min="4" max="4" width="29.5" style="10" customWidth="1"/>
     <col min="5" max="5" width="28.5" style="10" customWidth="1"/>
-    <col min="6" max="6" width="18.09765625" style="10" customWidth="1"/>
-    <col min="7" max="7" width="19.3984375" style="10" customWidth="1"/>
+    <col min="6" max="6" width="18.125" style="10" customWidth="1"/>
+    <col min="7" max="7" width="19.375" style="10" customWidth="1"/>
     <col min="8" max="16384" width="9" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="12" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B1" s="14">
-        <v>46207</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>46330</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D2" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="E2" s="11"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D3" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="E3" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="E2" s="11"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D3" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D4" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D5" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D6" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="E6" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="E4" s="13" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D5" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D6" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:7" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
@@ -2310,7 +2358,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="15" x14ac:dyDescent="0.2">
       <c r="B9" s="29" t="s">
         <v>31</v>
       </c>
@@ -2320,7 +2368,7 @@
       <c r="F9" s="30"/>
       <c r="G9" s="31"/>
     </row>
-    <row r="10" spans="1:7" ht="76.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="76.349999999999994" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="22">
         <v>1</v>
       </c>
@@ -2337,10 +2385,10 @@
         <v>40</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="66" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="76.5" x14ac:dyDescent="0.2">
       <c r="B11" s="18">
         <v>1.1000000000000001</v>
       </c>
@@ -2360,7 +2408,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="B12" s="18">
         <v>1.2</v>
       </c>
@@ -2380,7 +2428,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="76.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="76.349999999999994" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="18">
         <v>1.3</v>
       </c>
@@ -2400,7 +2448,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="18">
         <v>2</v>
       </c>
@@ -2420,7 +2468,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="96.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="96.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="18">
         <v>2.1</v>
       </c>
@@ -2440,7 +2488,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="132" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="127.5" x14ac:dyDescent="0.2">
       <c r="B16" s="18">
         <v>2.2000000000000002</v>
       </c>
@@ -2460,7 +2508,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="123" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" ht="123" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="18">
         <v>2.2999999999999998</v>
       </c>
@@ -2480,7 +2528,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="123.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" ht="123.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="18">
         <v>2.4</v>
       </c>
@@ -2500,7 +2548,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="145.19999999999999" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="153" x14ac:dyDescent="0.2">
       <c r="B19" s="18">
         <v>2.5</v>
       </c>
@@ -2520,7 +2568,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="105.6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" ht="114.75" x14ac:dyDescent="0.2">
       <c r="B20" s="18">
         <v>3</v>
       </c>
@@ -2540,7 +2588,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="105.6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" ht="114.75" x14ac:dyDescent="0.2">
       <c r="B21" s="18">
         <v>3.1</v>
       </c>
@@ -2560,7 +2608,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="59.4" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" ht="59.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="18">
         <v>3.2</v>
       </c>
@@ -2580,7 +2628,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="150" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" ht="150" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="18">
         <v>4</v>
       </c>
@@ -2600,7 +2648,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="79.2" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" ht="76.5" x14ac:dyDescent="0.2">
       <c r="B24" s="18">
         <v>5</v>
       </c>
@@ -2620,7 +2668,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="92.4" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" ht="102" x14ac:dyDescent="0.2">
       <c r="B25" s="18">
         <v>5.0999999999999996</v>
       </c>
@@ -2640,7 +2688,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" ht="51" x14ac:dyDescent="0.2">
       <c r="B26" s="18">
         <v>6</v>
       </c>
@@ -2657,10 +2705,10 @@
         <v>110</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="27" spans="2:7" ht="52.8" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" ht="51" x14ac:dyDescent="0.2">
       <c r="B27" s="18">
         <v>6.1</v>
       </c>
@@ -2677,90 +2725,90 @@
         <v>108</v>
       </c>
       <c r="G27" s="21" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="28" spans="2:7" ht="66" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" ht="63.75" x14ac:dyDescent="0.2">
       <c r="B28" s="18">
         <v>7</v>
       </c>
       <c r="C28" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="F28" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="G28" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="D28" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>154</v>
-      </c>
-      <c r="F28" s="21" t="s">
-        <v>155</v>
-      </c>
-      <c r="G28" s="21" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7" ht="66" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="2:7" ht="63.75" x14ac:dyDescent="0.2">
       <c r="B29" s="18">
         <v>7.1</v>
       </c>
       <c r="C29" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>154</v>
+      </c>
+      <c r="E29" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="D29" s="21" t="s">
-        <v>158</v>
-      </c>
-      <c r="E29" s="21" t="s">
-        <v>161</v>
-      </c>
       <c r="F29" s="21" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="G29" s="21" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="30" spans="2:7" ht="66" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="63.75" x14ac:dyDescent="0.2">
       <c r="B30" s="18">
         <v>7.2</v>
       </c>
       <c r="C30" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="D30" s="21" t="s">
+        <v>159</v>
+      </c>
+      <c r="E30" s="21" t="s">
+        <v>160</v>
+      </c>
+      <c r="F30" s="21" t="s">
+        <v>161</v>
+      </c>
+      <c r="G30" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="D30" s="21" t="s">
-        <v>163</v>
-      </c>
-      <c r="E30" s="21" t="s">
-        <v>164</v>
-      </c>
-      <c r="F30" s="21" t="s">
-        <v>165</v>
-      </c>
-      <c r="G30" s="21" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="31" spans="2:7" ht="66" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="2:7" ht="63.75" x14ac:dyDescent="0.2">
       <c r="B31" s="18">
         <v>7.3</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E31" s="21" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F31" s="21" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="G31" s="21" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="32" spans="2:7" ht="52.8" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" ht="51" x14ac:dyDescent="0.2">
       <c r="B32" s="18">
         <v>8</v>
       </c>
@@ -2780,100 +2828,160 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:7" ht="63.75" x14ac:dyDescent="0.2">
       <c r="B33" s="18">
+        <v>8.1</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>182</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>183</v>
+      </c>
+      <c r="E33" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="F33" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="G33" s="21" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="B34" s="18">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C34" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="D34" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="E34" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="F34" s="21" t="s">
+        <v>190</v>
+      </c>
+      <c r="G34" s="21" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="B35" s="18">
         <v>9</v>
       </c>
-      <c r="C33" s="21" t="s">
+      <c r="C35" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="D35" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="E35" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="F35" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="G35" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="D33" s="21" t="s">
+    </row>
+    <row r="36" spans="2:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="B36" s="18">
+        <v>9.1</v>
+      </c>
+      <c r="C36" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="E33" s="21" t="s">
+      <c r="D36" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="F33" s="21" t="s">
+      <c r="E36" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="G33" s="21" t="s">
+      <c r="F36" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="G36" s="21" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="B34" s="18">
-        <v>9.1</v>
-      </c>
-      <c r="C34" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="D34" s="21" t="s">
+    <row r="37" spans="2:7" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="B37" s="18">
+        <v>10</v>
+      </c>
+      <c r="C37" s="21" t="s">
         <v>177</v>
       </c>
-      <c r="E34" s="21" t="s">
+      <c r="D37" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="F34" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="G34" s="21" t="s">
+      <c r="E37" s="21" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="35" spans="2:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="B35" s="32" t="s">
+      <c r="F37" s="21" t="s">
+        <v>180</v>
+      </c>
+      <c r="G37" s="21" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="B38" s="32" t="s">
         <v>121</v>
       </c>
-      <c r="C35" s="32"/>
-      <c r="D35" s="32"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-    </row>
-    <row r="36" spans="2:7" ht="96" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="18">
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+    </row>
+    <row r="39" spans="2:7" ht="96" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B39" s="18">
         <v>1</v>
       </c>
-      <c r="C36" s="21" t="s">
+      <c r="C39" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="D39" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="E36" s="21" t="s">
+      <c r="E39" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="F36" s="21" t="s">
+      <c r="F39" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="G36" s="21" t="s">
+      <c r="G39" s="21" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="92.4" x14ac:dyDescent="0.25">
-      <c r="B37" s="18">
+    <row r="40" spans="2:7" ht="102" x14ac:dyDescent="0.2">
+      <c r="B40" s="18">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C37" s="21" t="s">
+      <c r="C40" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="D40" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="E37" s="21" t="s">
+      <c r="E40" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="F37" s="21" t="s">
+      <c r="F40" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="G37" s="21" t="s">
+      <c r="G40" s="21" t="s">
         <v>126</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B9:G9"/>
-    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B38:G38"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E6" r:id="rId1" xr:uid="{D85FBC9F-E10B-47AF-B754-81AB8B289351}"/>

</xml_diff>